<commit_message>
HQ: state park facilities from our saved layer (chat 3); agent sheet cut to the 70 other KY parks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015sd9rGiF55g53SvUATRP26
</commit_message>
<xml_diff>
--- a/.claude/build/research/KPC_Park_Facilities_worklist.xlsx
+++ b/.claude/build/research/KPC_Park_Facilities_worklist.xlsx
@@ -487,7 +487,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KPC park facilities for activators: Kentucky parks</t>
+          <t>KPC park facilities for activators: the Kentucky parks the state park map does NOT cover (nature preserves, forests, national sites)</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -697,12 +697,12 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>US-1273</t>
+          <t>US-1252</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Barren River Lake State Park</t>
+          <t>Columbus Belmont State Park</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/lucas/parks/resort/barren-river-lake-state-resort-park</t>
+          <t>https://parks.ky.gov/columbus/parks/historic/columbus-belmont-state-park</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr"/>
@@ -727,12 +727,12 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>US-1274</t>
+          <t>US-1278</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Blue Licks Battlefield State Park</t>
+          <t>Dale Hollow State Park</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/carlisle/parks/historic/blue-licks-battlefield-state-resort-park</t>
+          <t>https://parks.ky.gov/burkesville/parks/resort/dale-hollow-lake-state-resort-park</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr"/>
@@ -757,12 +757,12 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>US-3781</t>
+          <t>US-1254</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Breaks Interstate State Park</t>
+          <t>E.P. 'Tom' Sawyer State Park</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>https://www.breakspark.com/</t>
+          <t>https://parks.ky.gov/explore/e-p-tom-sawyer-state-park-7810</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
@@ -787,12 +787,12 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>US-1275</t>
+          <t>US-1264</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Buckhorn Lake State Park</t>
+          <t>Levi Jackson Wilderness Road State Park</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>https://next.pota.app/park/US-1275</t>
+          <t>https://levijacksonpark.com/</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
@@ -817,22 +817,22 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>US-1251</t>
+          <t>US-0724</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Carr Creek State Park</t>
+          <t>Abraham Lincoln Birthplace National Historic Site</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>https://next.pota.app/park/US-1251</t>
+          <t>https://www.nps.gov/abli/index.htm</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
@@ -847,22 +847,22 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>US-1276</t>
+          <t>US-10112</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Carter Caves State Park</t>
+          <t>Bad Branch National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/olive-hill/parks/resort/carter-caves-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Bad-Branch-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
@@ -877,22 +877,22 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>US-1252</t>
+          <t>US-10107</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Columbus Belmont State Park</t>
+          <t>Big South Fork National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/columbus/parks/historic/columbus-belmont-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Big-South-Fork-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr"/>
@@ -907,22 +907,22 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>US-1277</t>
+          <t>US-7950</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Cumberland Falls State Park</t>
+          <t>Camp Nelson National Monument</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/corbin/parks/resort/cumberland-falls-state-resort-park</t>
+          <t>https://www.nps.gov/cane/index.htm</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
@@ -937,22 +937,22 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>US-1278</t>
+          <t>US-0295</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Dale Hollow State Park</t>
+          <t>Clarks River National Wildlife Refuge</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/burkesville/parks/resort/dale-hollow-lake-state-resort-park</t>
+          <t>https://www.fws.gov/refuge/clarks-river</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr"/>
@@ -967,22 +967,22 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>US-1254</t>
+          <t>US-0019</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>E.P. 'Tom' Sawyer State Park</t>
+          <t>Cumberland Gap National Historical Park</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/explore/e-p-tom-sawyer-state-park-7810</t>
+          <t>https://www.nps.gov/cuga/index.htm</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
@@ -997,22 +997,22 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>US-1256</t>
+          <t>US-0703</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Fort Boonesborough State Park</t>
+          <t>Fort Donelson National Battlefield</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/richmond/parks/historic/fort-boonesborough-state-park</t>
+          <t>https://next.pota.app/park/US-0703</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
@@ -1027,22 +1027,22 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>US-1257</t>
+          <t>US-3790</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>General Burnside State Park</t>
+          <t>Fort Heiman National Battlefield</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/burnside/parks/recreation/general-burnside-island-state-park</t>
+          <t>https://www.nps.gov/fodo/planyourvisit/maps.htm</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
@@ -1057,22 +1057,22 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>US-1279</t>
+          <t>US-10098</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>General Butler State Park</t>
+          <t>Green River National Wildlife Refuge</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/carrollton/parks/historic/general-butler-state-resort-park</t>
+          <t>https://www.fws.gov/refuge/green-river/visit-us/locations/green-river-national-wildlife-refuge</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr"/>
@@ -1087,22 +1087,22 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>US-1258</t>
+          <t>US-4572</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Grayson Lake State Park</t>
+          <t>Lewis and Clark National Historic Trail</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/olive-hill/parks/recreation/grayson-lake-state-park</t>
+          <t>https://www.nps.gov/lecl/index.htm</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr"/>
@@ -1117,22 +1117,22 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>US-1259</t>
+          <t>US-7708</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Green River Lake State Park</t>
+          <t>Mill Springs Battlefield National Monument</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/campbellsville/parks/recreation/green-river-lake-state-park</t>
+          <t>https://www.nps.gov/misp/index.htm</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr"/>
@@ -1147,22 +1147,22 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>US-1280</t>
+          <t>US-0608</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Greenbo Lake State Park</t>
+          <t>Ohio River Islands National Wildlife Refuge</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/ashland/parks/historic/greenbo-lake-state-resort-park</t>
+          <t>https://www.fws.gov/refuge/ohio-river-islands</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr"/>
@@ -1177,22 +1177,22 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>US-1281</t>
+          <t>US-10104</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Jenny Wiley State Park</t>
+          <t>Red River National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/prestonsburg/parks/resort/jenny-wiley-state-resort-park</t>
+          <t>https://www.fs.usda.gov/recarea/dbnf/recreation/recarea/?recid=39548</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr"/>
@@ -1207,22 +1207,22 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>US-1260</t>
+          <t>US-0538</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>John James Audubon State Park</t>
+          <t>Reelfoot National Wildlife Refuge</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/henderson/parks/historic/john-james-audubon-state-park</t>
+          <t>https://www.fws.gov/refuge/reelfoot/</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr"/>
@@ -1237,22 +1237,22 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>US-1282</t>
+          <t>US-10111</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Kenlake State Park</t>
+          <t>Rock Creek National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/hardin/parks/resort/kenlake-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rock-Creek-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr"/>
@@ -1267,22 +1267,22 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>US-1283</t>
+          <t>US-10105</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Kentucky Dam Village State Park</t>
+          <t>The Green National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/gilbertsville/parks/resort/kentucky-dam-village-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Green-River-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr"/>
@@ -1297,22 +1297,22 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>US-1261</t>
+          <t>US-10106</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Kincaid Lake State Park</t>
+          <t>The Rockcastle National Wild and Scenic River</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/falmouth/parks/recreation/kincaid-lake-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rockcastle-River-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr"/>
@@ -1327,22 +1327,22 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>US-1262</t>
+          <t>US-3791</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Kingdom Come State Park</t>
+          <t>Trail of Tears National Historic Trail</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National / NPS</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/cumberland/parks/recreation/kingdom-come-state-park</t>
+          <t>https://www.nps.gov/trte/index.htm</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr"/>
@@ -1357,22 +1357,22 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>US-1284</t>
+          <t>US-0050</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Lake Barkley State Park</t>
+          <t>Mammoth Cave National Park</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National Park</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/cadiz/parks/resort/lake-barkley-state-resort-park</t>
+          <t>https://www.nps.gov/maca/index.htm</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr"/>
@@ -1387,22 +1387,22 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>US-1285</t>
+          <t>US-10172</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Lake Cumberland State Park</t>
+          <t>Salato Wildlife Refuge</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/jamestown/parks/resort/lake-cumberland-state-resort-park</t>
+          <t>https://fw.ky.gov/Education/Pages/Salato-Wildlife-Education-Center.aspx</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr"/>
@@ -1417,22 +1417,22 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>US-1263</t>
+          <t>US-3787</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Lake Malone State Park</t>
+          <t>White Hall State Historic Site</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/dunmor/parks/recreation/lake-malone-state-park</t>
+          <t>https://whitehall.eku.edu</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr"/>
@@ -1447,22 +1447,22 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>US-1264</t>
+          <t>US-3789</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Levi Jackson Wilderness Road State Park</t>
+          <t>William Whitley House State Historic Site</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>https://levijacksonpark.com/</t>
+          <t>https://explorekyhistory.ky.gov/files/show/236</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr"/>
@@ -1477,22 +1477,22 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>US-1265</t>
+          <t>US-8144</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Lincoln Homestead State Park</t>
+          <t>Otter Creek State Recreation Area</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Recreation Area</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/springfield/parks/historic/lincoln-homestead-state-park</t>
+          <t>https://fw.ky.gov/Pages/Otter-Creek-Outdoor-Recreation-Area.aspx</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr"/>
@@ -1507,22 +1507,22 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>US-1266</t>
+          <t>US-0686</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Mineral Mounds State Park</t>
+          <t>Big South Fork National Recreation Area</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National Recreation Area</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/eddyville/parks/recreation/mineral-mound-state-park</t>
+          <t>https://www.nps.gov/biso/index.htm</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr"/>
@@ -1537,22 +1537,22 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>US-1267</t>
+          <t>US-3792</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>My Old Kentucky Home State Park</t>
+          <t>Land Between the Lakes National Recreation Area</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>National Recreation Area</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/bardstown/parks/historic/my-old-kentucky-home-state-park</t>
+          <t>https://landbetweenthelakes.us/</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr"/>
@@ -1567,22 +1567,22 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>US-1286</t>
+          <t>US-7966</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Natural Bridge State Park</t>
+          <t>Bad Branch State Nature Preserve</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/slade/parks/resort/natural-bridge-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Bad-Branch.aspx</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr"/>
@@ -1597,22 +1597,22 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>US-1268</t>
+          <t>US-12971</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Nolin Lake State Park</t>
+          <t>Bat Cave State Nature Preserve</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/mammoth-cave/parks/recreation/nolin-lake-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Carter-Caves.aspx</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr"/>
@@ -1627,22 +1627,22 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>US-1269</t>
+          <t>US-7956</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Old Fort Harrod State Park</t>
+          <t>Beargrass Creek State Nature Preserve</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/harrodsburg/parks/historic/old-fort-harrod-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Beargrass-Creek.aspx</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr"/>
@@ -1657,22 +1657,22 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>US-1270</t>
+          <t>US-7954</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Paintsville Lake State Park</t>
+          <t>Blackacre State Nature Preserve</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/staffordsville/parks/recreation/paintsville-lake-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blackacre.aspx</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr"/>
@@ -1687,22 +1687,22 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>US-1287</t>
+          <t>US-7967</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Pennyrile Forest State Park</t>
+          <t>Blanton Forest State Nature Preserve</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/dawson-springs/parks/resort/pennyrile-forest-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blanton-Forest.aspx</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr"/>
@@ -1717,22 +1717,22 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>US-1288</t>
+          <t>US-7965</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Pine Mountain State Park</t>
+          <t>Brigadoon State Nature Preserve</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/pineville/parks/resort/pine-mountain-state-resort-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Brigadoon.aspx</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr"/>
@@ -1747,22 +1747,22 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>US-1289</t>
+          <t>US-12972</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Rough River Dam State Park</t>
+          <t>Cascade Caverns State Nature Preserve</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/falls-rough/parks/resort/rough-river-dam-state-resort-park</t>
+          <t>https://opengisdata.ky.gov/datasets/ky-knp-state-nature-preserves/explore?location=38.354945%2C-83.108279%2C14.97</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr"/>
@@ -1777,22 +1777,22 @@
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>US-1271</t>
+          <t>US-7960</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Taylorsville Lake State Park</t>
+          <t>Crooked Creek State Nature Preserve</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/mount-eden/parks/recreation/taylorsville-lake-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Crooked-Creek.aspx</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr"/>
@@ -1807,22 +1807,22 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>US-1272</t>
+          <t>US-7968</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Yatesville Lake State Park</t>
+          <t>E. Lucy Braun State Nature Preserve</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>State Park</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/louisa/parks/recreation/yatesville-lake-state-park</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/E.-Lucy-Braun.aspx</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr"/>
@@ -1837,22 +1837,22 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>US-0724</t>
+          <t>US-12752</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Abraham Lincoln Birthplace National Historic Site</t>
+          <t>Green River State Natural Area</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/abli/index.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rush-Island-Bottoms.aspx</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr"/>
@@ -1867,22 +1867,22 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>US-10112</t>
+          <t>US-7957</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Bad Branch National Wild and Scenic River</t>
+          <t>Hall-Hill/Vernon-Douglas State Nature Preserve</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Bad-Branch-Wild-River.aspx</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Vernon-Douglas.aspx</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr"/>
@@ -1897,22 +1897,22 @@
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>US-10107</t>
+          <t>US-7961</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Big South Fork National Wild and Scenic River</t>
+          <t>Jesse Stuart State Nature Preserve</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Big-South-Fork-Wild-River.aspx</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Jesse-Stuart.aspx</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr"/>
@@ -1927,22 +1927,22 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>US-7950</t>
+          <t>US-7958</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Camp Nelson National Monument</t>
+          <t>Kentucky River Palisades/Tom Dorman State Nature Preserve</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/cane/index.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Tom-Dorman.aspx</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>US-0295</t>
+          <t>US-7962</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Clarks River National Wildlife Refuge</t>
+          <t>Little South Fork State Natural Area</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>https://www.fws.gov/refuge/clarks-river</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Burnett-WWCA.aspx</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr"/>
@@ -1987,22 +1987,22 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>US-0019</t>
+          <t>US-7953</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Cumberland Gap National Historical Park</t>
+          <t>Metropolis Lake State Nature Preserve</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/cuga/index.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Metropolis-Lake.aspx</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr"/>
@@ -2017,22 +2017,22 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>US-0703</t>
+          <t>US-7963</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Fort Donelson National Battlefield</t>
+          <t>Pilot Knob State Nature Preserve</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>https://next.pota.app/park/US-0703</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Pilot-Knob.aspx</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr"/>
@@ -2047,22 +2047,22 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>US-3790</t>
+          <t>US-7959</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Fort Heiman National Battlefield</t>
+          <t>Quiet Trails State Nature Preserve</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/fodo/planyourvisit/maps.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Quiet-Trails.aspx</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr"/>
@@ -2077,22 +2077,22 @@
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>US-10098</t>
+          <t>US-7970</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Green River National Wildlife Refuge</t>
+          <t>Sinking Creek State Natural Area</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>https://www.fws.gov/refuge/green-river/visit-us/locations/green-river-national-wildlife-refuge</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Sinking-Creek.aspx</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr"/>
@@ -2107,22 +2107,22 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>US-4572</t>
+          <t>US-7955</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Lewis and Clark National Historic Trail</t>
+          <t>Six Mile Island State Nature Preserve</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/lecl/index.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Six-Mile-Island.aspx</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr"/>
@@ -2137,22 +2137,22 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>US-7708</t>
+          <t>US-7964</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Mill Springs Battlefield National Monument</t>
+          <t>William H. Martin State Natural Area</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>Nature Preserve</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/misp/index.htm</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Dr.-William-H.-Martin-WWCA.aspx</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr"/>
@@ -2167,22 +2167,22 @@
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>US-0608</t>
+          <t>US-7951</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Ohio River Islands National Wildlife Refuge</t>
+          <t>Green River State Forest</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>https://www.fws.gov/refuge/ohio-river-islands</t>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Green-River-State-Forest.aspx</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr"/>
@@ -2197,22 +2197,22 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>US-10104</t>
+          <t>US-4688</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Red River National Wild and Scenic River</t>
+          <t>Kentenia State Forest</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>https://www.fs.usda.gov/recarea/dbnf/recreation/recarea/?recid=39548</t>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentenia-State-Forest.aspx</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr"/>
@@ -2227,22 +2227,22 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>US-0538</t>
+          <t>US-4689</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Reelfoot National Wildlife Refuge</t>
+          <t>Kentucky Ridge State Forest</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>https://www.fws.gov/refuge/reelfoot/</t>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentucky-Ridge-State-Forest.aspx</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr"/>
@@ -2257,22 +2257,22 @@
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>US-10111</t>
+          <t>US-4690</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Rock Creek National Wild and Scenic River</t>
+          <t>Knobs State Forest</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rock-Creek-Wild-River.aspx</t>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Knobs-State-Forest-and-Wildlife-Management-Area.aspx</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr"/>
@@ -2287,22 +2287,22 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>US-10105</t>
+          <t>US-7952</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>The Green National Wild and Scenic River</t>
+          <t>Marrowbone State Forest</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Green-River-Wild-River.aspx</t>
+          <t>https://fw.ky.gov/More/Documents/MarrowboneStateForestandWMA_ALL.pdf</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr"/>
@@ -2317,22 +2317,22 @@
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>US-10106</t>
+          <t>US-4692</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>The Rockcastle National Wild and Scenic River</t>
+          <t>Pennyrile State Forest</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rockcastle-River-Wild-River.aspx</t>
+          <t>https://parks.ky.gov/dawson-springs/parks/resort/pennyrile-forest-state-resort-park</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr"/>
@@ -2347,22 +2347,22 @@
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>US-3791</t>
+          <t>US-4693</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Trail of Tears National Historic Trail</t>
+          <t>Tygarts State Forest</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>National / NPS</t>
+          <t>State Forest</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/trte/index.htm</t>
+          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Tygarts-State-Forest.aspx</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr"/>
@@ -2377,22 +2377,22 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>US-0050</t>
+          <t>US-11181</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Mammoth Cave National Park</t>
+          <t>Sheltowee Trace National Recreation Trail</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>National Park</t>
+          <t>Trail</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/maca/index.htm</t>
+          <t>https://www.fs.usda.gov/wildflowers/regions/southern/SheltoweeTrace/index.shtml</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr"/>
@@ -2407,22 +2407,22 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>US-3779</t>
+          <t>US-13598</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Big Bone Lick State Historic Site</t>
+          <t>Beaver Lake State Fishing Lake</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/union/parks/historic/big-bone-lick-state-historic-site</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=49</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr"/>
@@ -2437,22 +2437,22 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>US-3782</t>
+          <t>US-13607</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Dr. Thomas Walker State Historic Site</t>
+          <t>Boltz State Fishing Lake</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/barbourville/parks/historic/dr-thomas-walker-state-historic-site</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=50</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr"/>
@@ -2467,22 +2467,22 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>US-7890</t>
+          <t>US-13606</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Isaac Shelby Cemetery State Historic Site</t>
+          <t>Bullock Pen State Fishing Lake</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>https://next.pota.app/park/US-7890</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=51</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr"/>
@@ -2497,22 +2497,22 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>US-3783</t>
+          <t>US-13600</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Jefferson Davis State Historic Site</t>
+          <t>Carpenters Lake State Fishing Lake</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/fairview/parks/historic/jefferson-davis-state-historic-site</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=39</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr"/>
@@ -2527,22 +2527,22 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>US-3784</t>
+          <t>US-3801</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Old Mulkey Meetinghouse State Historic Site</t>
+          <t>Clifty Wilderness Area</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>River / Wilderness</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/tompkinsville/parks/historic/old-mulkey-meetinghouse-state-historic-site</t>
+          <t>https://www.fs.usda.gov/recarea/dbnf/recarea/?recid=39460</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr"/>
@@ -2557,22 +2557,22 @@
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>US-3785</t>
+          <t>US-3802</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Perryville Battlefield State Historic Site</t>
+          <t>Clyde E Buckley Sanctuary</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Sanctuary</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/perryville/parks/historic/perryville-battlefield-state-historic-site</t>
+          <t>https://bggreensource.org/buckley/</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr"/>
@@ -2587,22 +2587,22 @@
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>US-10172</t>
+          <t>US-4484</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Salato Wildlife Refuge</t>
+          <t>Daniel Boone National Forest</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>National Forest</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>https://fw.ky.gov/Education/Pages/Salato-Wildlife-Education-Center.aspx</t>
+          <t>https://www.fs.usda.gov/dbnf/</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr"/>
@@ -2617,22 +2617,22 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>US-3786</t>
+          <t>US-4526</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Waveland State Historic Site</t>
+          <t>George Washington &amp; Jefferson National Forest</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>National Forest</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/lexington/parks/historic/waveland-state-historic-site</t>
+          <t>https://www.fs.usda.gov/gwj</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr"/>
@@ -2647,22 +2647,22 @@
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>US-3787</t>
+          <t>US-13601</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>White Hall State Historic Site</t>
+          <t>Guist Creek Lake State Fishing Lake</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>https://whitehall.eku.edu</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=56</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr"/>
@@ -2677,22 +2677,22 @@
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>US-3788</t>
+          <t>US-10173</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Wickliffe Mounds State Historic Site</t>
+          <t>Kentucky Horse Park</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Facility</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>https://parks.ky.gov/wickliffe/parks/historic/wickliffe-mounds-state-historic-site</t>
+          <t>https://www.kyhorsepark.com/</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr"/>
@@ -2707,22 +2707,22 @@
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>US-3789</t>
+          <t>US-13599</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>William Whitley House State Historic Site</t>
+          <t>Kingfisher Lakes State Fishing Lake</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>State Fishing Lake</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>https://explorekyhistory.ky.gov/files/show/236</t>
+          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=40</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr"/>
@@ -2737,22 +2737,22 @@
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>US-8144</t>
+          <t>US-10103</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Otter Creek State Recreation Area</t>
+          <t>The Cumberland River Wilderness Area</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Recreation Area</t>
+          <t>River / Wilderness</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>https://fw.ky.gov/Pages/Otter-Creek-Outdoor-Recreation-Area.aspx</t>
+          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Cumberland-River-Wild-River.aspx</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr"/>
@@ -2767,22 +2767,22 @@
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>US-0686</t>
+          <t>US-10099</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>Big South Fork National Recreation Area</t>
+          <t>Wolf Creek National Fish Hatchery</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>National Recreation Area</t>
+          <t>Fish Hatchery</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>https://www.nps.gov/biso/index.htm</t>
+          <t>https://www.fws.gov/fish-hatchery/wolf-creek/map</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr"/>
@@ -2794,1326 +2794,6 @@
       <c r="K72" s="8" t="inlineStr"/>
       <c r="L72" s="8" t="inlineStr"/>
     </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>US-3792</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="inlineStr">
-        <is>
-          <t>Land Between the Lakes National Recreation Area</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>National Recreation Area</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>https://landbetweenthelakes.us/</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr"/>
-      <c r="F73" s="8" t="inlineStr"/>
-      <c r="G73" s="8" t="inlineStr"/>
-      <c r="H73" s="8" t="inlineStr"/>
-      <c r="I73" s="8" t="inlineStr"/>
-      <c r="J73" s="8" t="inlineStr"/>
-      <c r="K73" s="8" t="inlineStr"/>
-      <c r="L73" s="8" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>US-7966</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>Bad Branch State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D74" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Bad-Branch.aspx</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr"/>
-      <c r="G74" s="8" t="inlineStr"/>
-      <c r="H74" s="8" t="inlineStr"/>
-      <c r="I74" s="8" t="inlineStr"/>
-      <c r="J74" s="8" t="inlineStr"/>
-      <c r="K74" s="8" t="inlineStr"/>
-      <c r="L74" s="8" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>US-12971</t>
-        </is>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>Bat Cave State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Carter-Caves.aspx</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr"/>
-      <c r="F75" s="8" t="inlineStr"/>
-      <c r="G75" s="8" t="inlineStr"/>
-      <c r="H75" s="8" t="inlineStr"/>
-      <c r="I75" s="8" t="inlineStr"/>
-      <c r="J75" s="8" t="inlineStr"/>
-      <c r="K75" s="8" t="inlineStr"/>
-      <c r="L75" s="8" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>US-7956</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
-        <is>
-          <t>Beargrass Creek State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Beargrass-Creek.aspx</t>
-        </is>
-      </c>
-      <c r="E76" s="8" t="inlineStr"/>
-      <c r="F76" s="8" t="inlineStr"/>
-      <c r="G76" s="8" t="inlineStr"/>
-      <c r="H76" s="8" t="inlineStr"/>
-      <c r="I76" s="8" t="inlineStr"/>
-      <c r="J76" s="8" t="inlineStr"/>
-      <c r="K76" s="8" t="inlineStr"/>
-      <c r="L76" s="8" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="7" t="inlineStr">
-        <is>
-          <t>US-7954</t>
-        </is>
-      </c>
-      <c r="B77" s="7" t="inlineStr">
-        <is>
-          <t>Blackacre State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C77" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blackacre.aspx</t>
-        </is>
-      </c>
-      <c r="E77" s="8" t="inlineStr"/>
-      <c r="F77" s="8" t="inlineStr"/>
-      <c r="G77" s="8" t="inlineStr"/>
-      <c r="H77" s="8" t="inlineStr"/>
-      <c r="I77" s="8" t="inlineStr"/>
-      <c r="J77" s="8" t="inlineStr"/>
-      <c r="K77" s="8" t="inlineStr"/>
-      <c r="L77" s="8" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t>US-7967</t>
-        </is>
-      </c>
-      <c r="B78" s="7" t="inlineStr">
-        <is>
-          <t>Blanton Forest State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Blanton-Forest.aspx</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="inlineStr"/>
-      <c r="F78" s="8" t="inlineStr"/>
-      <c r="G78" s="8" t="inlineStr"/>
-      <c r="H78" s="8" t="inlineStr"/>
-      <c r="I78" s="8" t="inlineStr"/>
-      <c r="J78" s="8" t="inlineStr"/>
-      <c r="K78" s="8" t="inlineStr"/>
-      <c r="L78" s="8" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>US-7965</t>
-        </is>
-      </c>
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Brigadoon State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C79" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Brigadoon.aspx</t>
-        </is>
-      </c>
-      <c r="E79" s="8" t="inlineStr"/>
-      <c r="F79" s="8" t="inlineStr"/>
-      <c r="G79" s="8" t="inlineStr"/>
-      <c r="H79" s="8" t="inlineStr"/>
-      <c r="I79" s="8" t="inlineStr"/>
-      <c r="J79" s="8" t="inlineStr"/>
-      <c r="K79" s="8" t="inlineStr"/>
-      <c r="L79" s="8" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>US-12972</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="inlineStr">
-        <is>
-          <t>Cascade Caverns State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C80" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>https://opengisdata.ky.gov/datasets/ky-knp-state-nature-preserves/explore?location=38.354945%2C-83.108279%2C14.97</t>
-        </is>
-      </c>
-      <c r="E80" s="8" t="inlineStr"/>
-      <c r="F80" s="8" t="inlineStr"/>
-      <c r="G80" s="8" t="inlineStr"/>
-      <c r="H80" s="8" t="inlineStr"/>
-      <c r="I80" s="8" t="inlineStr"/>
-      <c r="J80" s="8" t="inlineStr"/>
-      <c r="K80" s="8" t="inlineStr"/>
-      <c r="L80" s="8" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="7" t="inlineStr">
-        <is>
-          <t>US-7960</t>
-        </is>
-      </c>
-      <c r="B81" s="7" t="inlineStr">
-        <is>
-          <t>Crooked Creek State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C81" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Crooked-Creek.aspx</t>
-        </is>
-      </c>
-      <c r="E81" s="8" t="inlineStr"/>
-      <c r="F81" s="8" t="inlineStr"/>
-      <c r="G81" s="8" t="inlineStr"/>
-      <c r="H81" s="8" t="inlineStr"/>
-      <c r="I81" s="8" t="inlineStr"/>
-      <c r="J81" s="8" t="inlineStr"/>
-      <c r="K81" s="8" t="inlineStr"/>
-      <c r="L81" s="8" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="7" t="inlineStr">
-        <is>
-          <t>US-7968</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>E. Lucy Braun State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/E.-Lucy-Braun.aspx</t>
-        </is>
-      </c>
-      <c r="E82" s="8" t="inlineStr"/>
-      <c r="F82" s="8" t="inlineStr"/>
-      <c r="G82" s="8" t="inlineStr"/>
-      <c r="H82" s="8" t="inlineStr"/>
-      <c r="I82" s="8" t="inlineStr"/>
-      <c r="J82" s="8" t="inlineStr"/>
-      <c r="K82" s="8" t="inlineStr"/>
-      <c r="L82" s="8" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>US-12752</t>
-        </is>
-      </c>
-      <c r="B83" s="7" t="inlineStr">
-        <is>
-          <t>Green River State Natural Area</t>
-        </is>
-      </c>
-      <c r="C83" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Rush-Island-Bottoms.aspx</t>
-        </is>
-      </c>
-      <c r="E83" s="8" t="inlineStr"/>
-      <c r="F83" s="8" t="inlineStr"/>
-      <c r="G83" s="8" t="inlineStr"/>
-      <c r="H83" s="8" t="inlineStr"/>
-      <c r="I83" s="8" t="inlineStr"/>
-      <c r="J83" s="8" t="inlineStr"/>
-      <c r="K83" s="8" t="inlineStr"/>
-      <c r="L83" s="8" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t>US-7957</t>
-        </is>
-      </c>
-      <c r="B84" s="7" t="inlineStr">
-        <is>
-          <t>Hall-Hill/Vernon-Douglas State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C84" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Vernon-Douglas.aspx</t>
-        </is>
-      </c>
-      <c r="E84" s="8" t="inlineStr"/>
-      <c r="F84" s="8" t="inlineStr"/>
-      <c r="G84" s="8" t="inlineStr"/>
-      <c r="H84" s="8" t="inlineStr"/>
-      <c r="I84" s="8" t="inlineStr"/>
-      <c r="J84" s="8" t="inlineStr"/>
-      <c r="K84" s="8" t="inlineStr"/>
-      <c r="L84" s="8" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="7" t="inlineStr">
-        <is>
-          <t>US-7961</t>
-        </is>
-      </c>
-      <c r="B85" s="7" t="inlineStr">
-        <is>
-          <t>Jesse Stuart State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C85" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Jesse-Stuart.aspx</t>
-        </is>
-      </c>
-      <c r="E85" s="8" t="inlineStr"/>
-      <c r="F85" s="8" t="inlineStr"/>
-      <c r="G85" s="8" t="inlineStr"/>
-      <c r="H85" s="8" t="inlineStr"/>
-      <c r="I85" s="8" t="inlineStr"/>
-      <c r="J85" s="8" t="inlineStr"/>
-      <c r="K85" s="8" t="inlineStr"/>
-      <c r="L85" s="8" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>US-7958</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
-        <is>
-          <t>Kentucky River Palisades/Tom Dorman State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C86" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Tom-Dorman.aspx</t>
-        </is>
-      </c>
-      <c r="E86" s="8" t="inlineStr"/>
-      <c r="F86" s="8" t="inlineStr"/>
-      <c r="G86" s="8" t="inlineStr"/>
-      <c r="H86" s="8" t="inlineStr"/>
-      <c r="I86" s="8" t="inlineStr"/>
-      <c r="J86" s="8" t="inlineStr"/>
-      <c r="K86" s="8" t="inlineStr"/>
-      <c r="L86" s="8" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="7" t="inlineStr">
-        <is>
-          <t>US-7962</t>
-        </is>
-      </c>
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>Little South Fork State Natural Area</t>
-        </is>
-      </c>
-      <c r="C87" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Burnett-WWCA.aspx</t>
-        </is>
-      </c>
-      <c r="E87" s="8" t="inlineStr"/>
-      <c r="F87" s="8" t="inlineStr"/>
-      <c r="G87" s="8" t="inlineStr"/>
-      <c r="H87" s="8" t="inlineStr"/>
-      <c r="I87" s="8" t="inlineStr"/>
-      <c r="J87" s="8" t="inlineStr"/>
-      <c r="K87" s="8" t="inlineStr"/>
-      <c r="L87" s="8" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t>US-7953</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
-        <is>
-          <t>Metropolis Lake State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C88" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D88" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Metropolis-Lake.aspx</t>
-        </is>
-      </c>
-      <c r="E88" s="8" t="inlineStr"/>
-      <c r="F88" s="8" t="inlineStr"/>
-      <c r="G88" s="8" t="inlineStr"/>
-      <c r="H88" s="8" t="inlineStr"/>
-      <c r="I88" s="8" t="inlineStr"/>
-      <c r="J88" s="8" t="inlineStr"/>
-      <c r="K88" s="8" t="inlineStr"/>
-      <c r="L88" s="8" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
-        <is>
-          <t>US-7963</t>
-        </is>
-      </c>
-      <c r="B89" s="7" t="inlineStr">
-        <is>
-          <t>Pilot Knob State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C89" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Pilot-Knob.aspx</t>
-        </is>
-      </c>
-      <c r="E89" s="8" t="inlineStr"/>
-      <c r="F89" s="8" t="inlineStr"/>
-      <c r="G89" s="8" t="inlineStr"/>
-      <c r="H89" s="8" t="inlineStr"/>
-      <c r="I89" s="8" t="inlineStr"/>
-      <c r="J89" s="8" t="inlineStr"/>
-      <c r="K89" s="8" t="inlineStr"/>
-      <c r="L89" s="8" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="7" t="inlineStr">
-        <is>
-          <t>US-7959</t>
-        </is>
-      </c>
-      <c r="B90" s="7" t="inlineStr">
-        <is>
-          <t>Quiet Trails State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C90" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Quiet-Trails.aspx</t>
-        </is>
-      </c>
-      <c r="E90" s="8" t="inlineStr"/>
-      <c r="F90" s="8" t="inlineStr"/>
-      <c r="G90" s="8" t="inlineStr"/>
-      <c r="H90" s="8" t="inlineStr"/>
-      <c r="I90" s="8" t="inlineStr"/>
-      <c r="J90" s="8" t="inlineStr"/>
-      <c r="K90" s="8" t="inlineStr"/>
-      <c r="L90" s="8" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>US-7970</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="inlineStr">
-        <is>
-          <t>Sinking Creek State Natural Area</t>
-        </is>
-      </c>
-      <c r="C91" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Sinking-Creek.aspx</t>
-        </is>
-      </c>
-      <c r="E91" s="8" t="inlineStr"/>
-      <c r="F91" s="8" t="inlineStr"/>
-      <c r="G91" s="8" t="inlineStr"/>
-      <c r="H91" s="8" t="inlineStr"/>
-      <c r="I91" s="8" t="inlineStr"/>
-      <c r="J91" s="8" t="inlineStr"/>
-      <c r="K91" s="8" t="inlineStr"/>
-      <c r="L91" s="8" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>US-7955</t>
-        </is>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
-        <is>
-          <t>Six Mile Island State Nature Preserve</t>
-        </is>
-      </c>
-      <c r="C92" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Six-Mile-Island.aspx</t>
-        </is>
-      </c>
-      <c r="E92" s="8" t="inlineStr"/>
-      <c r="F92" s="8" t="inlineStr"/>
-      <c r="G92" s="8" t="inlineStr"/>
-      <c r="H92" s="8" t="inlineStr"/>
-      <c r="I92" s="8" t="inlineStr"/>
-      <c r="J92" s="8" t="inlineStr"/>
-      <c r="K92" s="8" t="inlineStr"/>
-      <c r="L92" s="8" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t>US-7964</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
-        <is>
-          <t>William H. Martin State Natural Area</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr">
-        <is>
-          <t>Nature Preserve</t>
-        </is>
-      </c>
-      <c r="D93" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Dr.-William-H.-Martin-WWCA.aspx</t>
-        </is>
-      </c>
-      <c r="E93" s="8" t="inlineStr"/>
-      <c r="F93" s="8" t="inlineStr"/>
-      <c r="G93" s="8" t="inlineStr"/>
-      <c r="H93" s="8" t="inlineStr"/>
-      <c r="I93" s="8" t="inlineStr"/>
-      <c r="J93" s="8" t="inlineStr"/>
-      <c r="K93" s="8" t="inlineStr"/>
-      <c r="L93" s="8" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t>US-7951</t>
-        </is>
-      </c>
-      <c r="B94" s="7" t="inlineStr">
-        <is>
-          <t>Green River State Forest</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D94" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Green-River-State-Forest.aspx</t>
-        </is>
-      </c>
-      <c r="E94" s="8" t="inlineStr"/>
-      <c r="F94" s="8" t="inlineStr"/>
-      <c r="G94" s="8" t="inlineStr"/>
-      <c r="H94" s="8" t="inlineStr"/>
-      <c r="I94" s="8" t="inlineStr"/>
-      <c r="J94" s="8" t="inlineStr"/>
-      <c r="K94" s="8" t="inlineStr"/>
-      <c r="L94" s="8" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="7" t="inlineStr">
-        <is>
-          <t>US-4688</t>
-        </is>
-      </c>
-      <c r="B95" s="7" t="inlineStr">
-        <is>
-          <t>Kentenia State Forest</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentenia-State-Forest.aspx</t>
-        </is>
-      </c>
-      <c r="E95" s="8" t="inlineStr"/>
-      <c r="F95" s="8" t="inlineStr"/>
-      <c r="G95" s="8" t="inlineStr"/>
-      <c r="H95" s="8" t="inlineStr"/>
-      <c r="I95" s="8" t="inlineStr"/>
-      <c r="J95" s="8" t="inlineStr"/>
-      <c r="K95" s="8" t="inlineStr"/>
-      <c r="L95" s="8" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t>US-4689</t>
-        </is>
-      </c>
-      <c r="B96" s="7" t="inlineStr">
-        <is>
-          <t>Kentucky Ridge State Forest</t>
-        </is>
-      </c>
-      <c r="C96" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Kentucky-Ridge-State-Forest.aspx</t>
-        </is>
-      </c>
-      <c r="E96" s="8" t="inlineStr"/>
-      <c r="F96" s="8" t="inlineStr"/>
-      <c r="G96" s="8" t="inlineStr"/>
-      <c r="H96" s="8" t="inlineStr"/>
-      <c r="I96" s="8" t="inlineStr"/>
-      <c r="J96" s="8" t="inlineStr"/>
-      <c r="K96" s="8" t="inlineStr"/>
-      <c r="L96" s="8" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>US-4690</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>Knobs State Forest</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Knobs-State-Forest-and-Wildlife-Management-Area.aspx</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr"/>
-      <c r="F97" s="8" t="inlineStr"/>
-      <c r="G97" s="8" t="inlineStr"/>
-      <c r="H97" s="8" t="inlineStr"/>
-      <c r="I97" s="8" t="inlineStr"/>
-      <c r="J97" s="8" t="inlineStr"/>
-      <c r="K97" s="8" t="inlineStr"/>
-      <c r="L97" s="8" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t>US-7952</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Marrowbone State Forest</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>https://fw.ky.gov/More/Documents/MarrowboneStateForestandWMA_ALL.pdf</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr"/>
-      <c r="F98" s="8" t="inlineStr"/>
-      <c r="G98" s="8" t="inlineStr"/>
-      <c r="H98" s="8" t="inlineStr"/>
-      <c r="I98" s="8" t="inlineStr"/>
-      <c r="J98" s="8" t="inlineStr"/>
-      <c r="K98" s="8" t="inlineStr"/>
-      <c r="L98" s="8" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="7" t="inlineStr">
-        <is>
-          <t>US-4692</t>
-        </is>
-      </c>
-      <c r="B99" s="7" t="inlineStr">
-        <is>
-          <t>Pennyrile State Forest</t>
-        </is>
-      </c>
-      <c r="C99" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t>https://parks.ky.gov/dawson-springs/parks/resort/pennyrile-forest-state-resort-park</t>
-        </is>
-      </c>
-      <c r="E99" s="8" t="inlineStr"/>
-      <c r="F99" s="8" t="inlineStr"/>
-      <c r="G99" s="8" t="inlineStr"/>
-      <c r="H99" s="8" t="inlineStr"/>
-      <c r="I99" s="8" t="inlineStr"/>
-      <c r="J99" s="8" t="inlineStr"/>
-      <c r="K99" s="8" t="inlineStr"/>
-      <c r="L99" s="8" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="7" t="inlineStr">
-        <is>
-          <t>US-4693</t>
-        </is>
-      </c>
-      <c r="B100" s="7" t="inlineStr">
-        <is>
-          <t>Tygarts State Forest</t>
-        </is>
-      </c>
-      <c r="C100" s="7" t="inlineStr">
-        <is>
-          <t>State Forest</t>
-        </is>
-      </c>
-      <c r="D100" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Natural-Resources/Forestry/ky-state-forests/Pages/Tygarts-State-Forest.aspx</t>
-        </is>
-      </c>
-      <c r="E100" s="8" t="inlineStr"/>
-      <c r="F100" s="8" t="inlineStr"/>
-      <c r="G100" s="8" t="inlineStr"/>
-      <c r="H100" s="8" t="inlineStr"/>
-      <c r="I100" s="8" t="inlineStr"/>
-      <c r="J100" s="8" t="inlineStr"/>
-      <c r="K100" s="8" t="inlineStr"/>
-      <c r="L100" s="8" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="7" t="inlineStr">
-        <is>
-          <t>US-1253</t>
-        </is>
-      </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>Dawkins Line Rail Trail State Park</t>
-        </is>
-      </c>
-      <c r="C101" s="7" t="inlineStr">
-        <is>
-          <t>Trail</t>
-        </is>
-      </c>
-      <c r="D101" s="7" t="inlineStr">
-        <is>
-          <t>https://parks.ky.gov/swamp-branch/parks/recreation/dawkins-line-rail-trail</t>
-        </is>
-      </c>
-      <c r="E101" s="8" t="inlineStr"/>
-      <c r="F101" s="8" t="inlineStr"/>
-      <c r="G101" s="8" t="inlineStr"/>
-      <c r="H101" s="8" t="inlineStr"/>
-      <c r="I101" s="8" t="inlineStr"/>
-      <c r="J101" s="8" t="inlineStr"/>
-      <c r="K101" s="8" t="inlineStr"/>
-      <c r="L101" s="8" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="7" t="inlineStr">
-        <is>
-          <t>US-10102</t>
-        </is>
-      </c>
-      <c r="B102" s="7" t="inlineStr">
-        <is>
-          <t>Pine Mountain State Trail</t>
-        </is>
-      </c>
-      <c r="C102" s="7" t="inlineStr">
-        <is>
-          <t>Trail</t>
-        </is>
-      </c>
-      <c r="D102" s="7" t="inlineStr">
-        <is>
-          <t>https://parks.ky.gov/whitesburg/parks/recreation/pine-mountain-state-scenic-trail</t>
-        </is>
-      </c>
-      <c r="E102" s="8" t="inlineStr"/>
-      <c r="F102" s="8" t="inlineStr"/>
-      <c r="G102" s="8" t="inlineStr"/>
-      <c r="H102" s="8" t="inlineStr"/>
-      <c r="I102" s="8" t="inlineStr"/>
-      <c r="J102" s="8" t="inlineStr"/>
-      <c r="K102" s="8" t="inlineStr"/>
-      <c r="L102" s="8" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="7" t="inlineStr">
-        <is>
-          <t>US-11181</t>
-        </is>
-      </c>
-      <c r="B103" s="7" t="inlineStr">
-        <is>
-          <t>Sheltowee Trace National Recreation Trail</t>
-        </is>
-      </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>Trail</t>
-        </is>
-      </c>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fs.usda.gov/wildflowers/regions/southern/SheltoweeTrace/index.shtml</t>
-        </is>
-      </c>
-      <c r="E103" s="8" t="inlineStr"/>
-      <c r="F103" s="8" t="inlineStr"/>
-      <c r="G103" s="8" t="inlineStr"/>
-      <c r="H103" s="8" t="inlineStr"/>
-      <c r="I103" s="8" t="inlineStr"/>
-      <c r="J103" s="8" t="inlineStr"/>
-      <c r="K103" s="8" t="inlineStr"/>
-      <c r="L103" s="8" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="7" t="inlineStr">
-        <is>
-          <t>US-13598</t>
-        </is>
-      </c>
-      <c r="B104" s="7" t="inlineStr">
-        <is>
-          <t>Beaver Lake State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C104" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D104" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=49</t>
-        </is>
-      </c>
-      <c r="E104" s="8" t="inlineStr"/>
-      <c r="F104" s="8" t="inlineStr"/>
-      <c r="G104" s="8" t="inlineStr"/>
-      <c r="H104" s="8" t="inlineStr"/>
-      <c r="I104" s="8" t="inlineStr"/>
-      <c r="J104" s="8" t="inlineStr"/>
-      <c r="K104" s="8" t="inlineStr"/>
-      <c r="L104" s="8" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="7" t="inlineStr">
-        <is>
-          <t>US-13607</t>
-        </is>
-      </c>
-      <c r="B105" s="7" t="inlineStr">
-        <is>
-          <t>Boltz State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=50</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr"/>
-      <c r="F105" s="8" t="inlineStr"/>
-      <c r="G105" s="8" t="inlineStr"/>
-      <c r="H105" s="8" t="inlineStr"/>
-      <c r="I105" s="8" t="inlineStr"/>
-      <c r="J105" s="8" t="inlineStr"/>
-      <c r="K105" s="8" t="inlineStr"/>
-      <c r="L105" s="8" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="7" t="inlineStr">
-        <is>
-          <t>US-13606</t>
-        </is>
-      </c>
-      <c r="B106" s="7" t="inlineStr">
-        <is>
-          <t>Bullock Pen State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C106" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=51</t>
-        </is>
-      </c>
-      <c r="E106" s="8" t="inlineStr"/>
-      <c r="F106" s="8" t="inlineStr"/>
-      <c r="G106" s="8" t="inlineStr"/>
-      <c r="H106" s="8" t="inlineStr"/>
-      <c r="I106" s="8" t="inlineStr"/>
-      <c r="J106" s="8" t="inlineStr"/>
-      <c r="K106" s="8" t="inlineStr"/>
-      <c r="L106" s="8" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>US-13600</t>
-        </is>
-      </c>
-      <c r="B107" s="7" t="inlineStr">
-        <is>
-          <t>Carpenters Lake State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=39</t>
-        </is>
-      </c>
-      <c r="E107" s="8" t="inlineStr"/>
-      <c r="F107" s="8" t="inlineStr"/>
-      <c r="G107" s="8" t="inlineStr"/>
-      <c r="H107" s="8" t="inlineStr"/>
-      <c r="I107" s="8" t="inlineStr"/>
-      <c r="J107" s="8" t="inlineStr"/>
-      <c r="K107" s="8" t="inlineStr"/>
-      <c r="L107" s="8" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="7" t="inlineStr">
-        <is>
-          <t>US-3801</t>
-        </is>
-      </c>
-      <c r="B108" s="7" t="inlineStr">
-        <is>
-          <t>Clifty Wilderness Area</t>
-        </is>
-      </c>
-      <c r="C108" s="7" t="inlineStr">
-        <is>
-          <t>River / Wilderness</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fs.usda.gov/recarea/dbnf/recarea/?recid=39460</t>
-        </is>
-      </c>
-      <c r="E108" s="8" t="inlineStr"/>
-      <c r="F108" s="8" t="inlineStr"/>
-      <c r="G108" s="8" t="inlineStr"/>
-      <c r="H108" s="8" t="inlineStr"/>
-      <c r="I108" s="8" t="inlineStr"/>
-      <c r="J108" s="8" t="inlineStr"/>
-      <c r="K108" s="8" t="inlineStr"/>
-      <c r="L108" s="8" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>US-3802</t>
-        </is>
-      </c>
-      <c r="B109" s="7" t="inlineStr">
-        <is>
-          <t>Clyde E Buckley Sanctuary</t>
-        </is>
-      </c>
-      <c r="C109" s="7" t="inlineStr">
-        <is>
-          <t>Sanctuary</t>
-        </is>
-      </c>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t>https://bggreensource.org/buckley/</t>
-        </is>
-      </c>
-      <c r="E109" s="8" t="inlineStr"/>
-      <c r="F109" s="8" t="inlineStr"/>
-      <c r="G109" s="8" t="inlineStr"/>
-      <c r="H109" s="8" t="inlineStr"/>
-      <c r="I109" s="8" t="inlineStr"/>
-      <c r="J109" s="8" t="inlineStr"/>
-      <c r="K109" s="8" t="inlineStr"/>
-      <c r="L109" s="8" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="7" t="inlineStr">
-        <is>
-          <t>US-4484</t>
-        </is>
-      </c>
-      <c r="B110" s="7" t="inlineStr">
-        <is>
-          <t>Daniel Boone National Forest</t>
-        </is>
-      </c>
-      <c r="C110" s="7" t="inlineStr">
-        <is>
-          <t>National Forest</t>
-        </is>
-      </c>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fs.usda.gov/dbnf/</t>
-        </is>
-      </c>
-      <c r="E110" s="8" t="inlineStr"/>
-      <c r="F110" s="8" t="inlineStr"/>
-      <c r="G110" s="8" t="inlineStr"/>
-      <c r="H110" s="8" t="inlineStr"/>
-      <c r="I110" s="8" t="inlineStr"/>
-      <c r="J110" s="8" t="inlineStr"/>
-      <c r="K110" s="8" t="inlineStr"/>
-      <c r="L110" s="8" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="7" t="inlineStr">
-        <is>
-          <t>US-4526</t>
-        </is>
-      </c>
-      <c r="B111" s="7" t="inlineStr">
-        <is>
-          <t>George Washington &amp; Jefferson National Forest</t>
-        </is>
-      </c>
-      <c r="C111" s="7" t="inlineStr">
-        <is>
-          <t>National Forest</t>
-        </is>
-      </c>
-      <c r="D111" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fs.usda.gov/gwj</t>
-        </is>
-      </c>
-      <c r="E111" s="8" t="inlineStr"/>
-      <c r="F111" s="8" t="inlineStr"/>
-      <c r="G111" s="8" t="inlineStr"/>
-      <c r="H111" s="8" t="inlineStr"/>
-      <c r="I111" s="8" t="inlineStr"/>
-      <c r="J111" s="8" t="inlineStr"/>
-      <c r="K111" s="8" t="inlineStr"/>
-      <c r="L111" s="8" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="7" t="inlineStr">
-        <is>
-          <t>US-13601</t>
-        </is>
-      </c>
-      <c r="B112" s="7" t="inlineStr">
-        <is>
-          <t>Guist Creek Lake State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C112" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D112" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=56</t>
-        </is>
-      </c>
-      <c r="E112" s="8" t="inlineStr"/>
-      <c r="F112" s="8" t="inlineStr"/>
-      <c r="G112" s="8" t="inlineStr"/>
-      <c r="H112" s="8" t="inlineStr"/>
-      <c r="I112" s="8" t="inlineStr"/>
-      <c r="J112" s="8" t="inlineStr"/>
-      <c r="K112" s="8" t="inlineStr"/>
-      <c r="L112" s="8" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="7" t="inlineStr">
-        <is>
-          <t>US-10173</t>
-        </is>
-      </c>
-      <c r="B113" s="7" t="inlineStr">
-        <is>
-          <t>Kentucky Horse Park</t>
-        </is>
-      </c>
-      <c r="C113" s="7" t="inlineStr">
-        <is>
-          <t>State Facility</t>
-        </is>
-      </c>
-      <c r="D113" s="7" t="inlineStr">
-        <is>
-          <t>https://www.kyhorsepark.com/</t>
-        </is>
-      </c>
-      <c r="E113" s="8" t="inlineStr"/>
-      <c r="F113" s="8" t="inlineStr"/>
-      <c r="G113" s="8" t="inlineStr"/>
-      <c r="H113" s="8" t="inlineStr"/>
-      <c r="I113" s="8" t="inlineStr"/>
-      <c r="J113" s="8" t="inlineStr"/>
-      <c r="K113" s="8" t="inlineStr"/>
-      <c r="L113" s="8" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="7" t="inlineStr">
-        <is>
-          <t>US-13599</t>
-        </is>
-      </c>
-      <c r="B114" s="7" t="inlineStr">
-        <is>
-          <t>Kingfisher Lakes State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="C114" s="7" t="inlineStr">
-        <is>
-          <t>State Fishing Lake</t>
-        </is>
-      </c>
-      <c r="D114" s="7" t="inlineStr">
-        <is>
-          <t>https://app.fw.ky.gov/fisheries/waterbodydetail.aspx?wid=40</t>
-        </is>
-      </c>
-      <c r="E114" s="8" t="inlineStr"/>
-      <c r="F114" s="8" t="inlineStr"/>
-      <c r="G114" s="8" t="inlineStr"/>
-      <c r="H114" s="8" t="inlineStr"/>
-      <c r="I114" s="8" t="inlineStr"/>
-      <c r="J114" s="8" t="inlineStr"/>
-      <c r="K114" s="8" t="inlineStr"/>
-      <c r="L114" s="8" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="7" t="inlineStr">
-        <is>
-          <t>US-10103</t>
-        </is>
-      </c>
-      <c r="B115" s="7" t="inlineStr">
-        <is>
-          <t>The Cumberland River Wilderness Area</t>
-        </is>
-      </c>
-      <c r="C115" s="7" t="inlineStr">
-        <is>
-          <t>River / Wilderness</t>
-        </is>
-      </c>
-      <c r="D115" s="7" t="inlineStr">
-        <is>
-          <t>https://eec.ky.gov/Nature-Preserves/Locations/Pages/Cumberland-River-Wild-River.aspx</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr"/>
-      <c r="F115" s="8" t="inlineStr"/>
-      <c r="G115" s="8" t="inlineStr"/>
-      <c r="H115" s="8" t="inlineStr"/>
-      <c r="I115" s="8" t="inlineStr"/>
-      <c r="J115" s="8" t="inlineStr"/>
-      <c r="K115" s="8" t="inlineStr"/>
-      <c r="L115" s="8" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="7" t="inlineStr">
-        <is>
-          <t>US-10099</t>
-        </is>
-      </c>
-      <c r="B116" s="7" t="inlineStr">
-        <is>
-          <t>Wolf Creek National Fish Hatchery</t>
-        </is>
-      </c>
-      <c r="C116" s="7" t="inlineStr">
-        <is>
-          <t>Fish Hatchery</t>
-        </is>
-      </c>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t>https://www.fws.gov/fish-hatchery/wolf-creek/map</t>
-        </is>
-      </c>
-      <c r="E116" s="8" t="inlineStr"/>
-      <c r="F116" s="8" t="inlineStr"/>
-      <c r="G116" s="8" t="inlineStr"/>
-      <c r="H116" s="8" t="inlineStr"/>
-      <c r="I116" s="8" t="inlineStr"/>
-      <c r="J116" s="8" t="inlineStr"/>
-      <c r="K116" s="8" t="inlineStr"/>
-      <c r="L116" s="8" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>